<commit_message>
Reporte actualizado automáticamente el 2026-04-29
</commit_message>
<xml_diff>
--- a/Programmes Seguimiento LE_2.xlsx
+++ b/Programmes Seguimiento LE_2.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364">
   <si>
     <t/>
   </si>
@@ -1099,6 +1099,15 @@
   </si>
   <si>
     <t>24:06:09</t>
+  </si>
+  <si>
+    <t>07:59:24</t>
+  </si>
+  <si>
+    <t>07:59:25</t>
+  </si>
+  <si>
+    <t>24:07:08</t>
   </si>
 </sst>
 </file>
@@ -1524,7 +1533,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H602"/>
+  <dimension ref="A2:H616"/>
   <sheetData>
     <row r="2" ht="15">
       <c r="A2" s="1" t="s">
@@ -15352,8 +15361,330 @@
         <v>840.397614</v>
       </c>
     </row>
+    <row r="603" ht="15">
+      <c r="A603" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B603" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C603" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D603" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E603" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="F603" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G603" s="5">
+        <v>952.984297</v>
+      </c>
+    </row>
+    <row r="604" ht="15">
+      <c r="A604" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B604" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C604" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D604" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="E604" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F604" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G604" s="5">
+        <v>1086.521685</v>
+      </c>
+    </row>
+    <row r="605" ht="15">
+      <c r="A605" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B605" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C605" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D605" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E605" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F605" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G605" s="5">
+        <v>1416.291135</v>
+      </c>
+    </row>
+    <row r="606" ht="15">
+      <c r="A606" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B606" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C606" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D606" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E606" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F606" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G606" s="5">
+        <v>1643.989937</v>
+      </c>
+    </row>
+    <row r="607" ht="15">
+      <c r="A607" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B607" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C607" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D607" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E607" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F607" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G607" s="5">
+        <v>1623.748738</v>
+      </c>
+    </row>
+    <row r="608" ht="15">
+      <c r="A608" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B608" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C608" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D608" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E608" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F608" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G608" s="5">
+        <v>2329.139386</v>
+      </c>
+    </row>
+    <row r="609" ht="15">
+      <c r="A609" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B609" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C609" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D609" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E609" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F609" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="G609" s="5">
+        <v>2668.204947</v>
+      </c>
+    </row>
+    <row r="610" ht="15">
+      <c r="A610" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B610" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C610" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D610" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E610" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F610" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="G610" s="5">
+        <v>3180.595386</v>
+      </c>
+    </row>
+    <row r="611" ht="15">
+      <c r="A611" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B611" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C611" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D611" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E611" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F611" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G611" s="5">
+        <v>3714.159851</v>
+      </c>
+    </row>
+    <row r="612" ht="15">
+      <c r="A612" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B612" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C612" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D612" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E612" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F612" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G612" s="5">
+        <v>4248.682222</v>
+      </c>
+    </row>
+    <row r="613" ht="15">
+      <c r="A613" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B613" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C613" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D613" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E613" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="F613" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G613" s="5">
+        <v>4408.283647</v>
+      </c>
+    </row>
+    <row r="614" ht="15">
+      <c r="A614" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B614" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C614" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D614" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="E614" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F614" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="G614" s="5">
+        <v>4163.167099</v>
+      </c>
+    </row>
+    <row r="615" ht="15">
+      <c r="A615" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B615" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C615" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D615" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E615" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="F615" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G615" s="5">
+        <v>2694.397996</v>
+      </c>
+    </row>
+    <row r="616" ht="15">
+      <c r="A616" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B616" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C616" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D616" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="E616" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F616" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G616" s="5">
+        <v>846.910185</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="5" fitToHeight="0" orientation="portrait"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reporte actualizado automaticamente el 2026-06-05
</commit_message>
<xml_diff>
--- a/Programmes Seguimiento LE_2.xlsx
+++ b/Programmes Seguimiento LE_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Seguimiento-LE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F722260F-E693-4B27-965A-73DD2D4EE26B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC12DA7A-673A-4F72-BD70-B0178B69318D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1836" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="69">
   <si>
     <t>Targets</t>
   </si>
@@ -170,7 +170,7 @@
     <t>Tv Programs</t>
   </si>
   <si>
-    <t>10/04/2026;   13/04/2026 - 17/04/2026;   20/04/2026 - 24/04/2026;   27/04/2026 - 01/05/2026;   04/05/2026 - 08/05/2026;   11/05/2026 - 15/05/2026;   18/05/2026 - 22/05/2026;   25/05/2026 - 29/05/2026;   01/06/2026 - 03/06/2026</t>
+    <t>10/04/2026;   13/04/2026 - 17/04/2026;   20/04/2026 - 24/04/2026;   27/04/2026 - 01/05/2026;   04/05/2026 - 08/05/2026;   11/05/2026 - 15/05/2026;   18/05/2026 - 22/05/2026;   25/05/2026 - 29/05/2026;   01/06/2026 - 04/06/2026</t>
   </si>
   <si>
     <t>National</t>
@@ -221,13 +221,13 @@
     <t xml:space="preserve">	For Target [P.2+] ...</t>
   </si>
   <si>
-    <t xml:space="preserve">	 For Region [National] Universe 78427.2; Sample 6882 ( 100.00% )</t>
+    <t xml:space="preserve">	 For Region [National] Universe 78427.2; Sample 6883 ( 100.00% )</t>
   </si>
   <si>
     <t xml:space="preserve">	For Target [Universe] ...</t>
   </si>
   <si>
-    <t xml:space="preserve">	 For Region [National] Universe 78427.2; Sample 6828 ( 100.00% )</t>
+    <t xml:space="preserve">	 For Region [National] Universe 78427.2; Sample 6829 ( 100.00% )</t>
   </si>
 </sst>
 </file>
@@ -769,7 +769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H597"/>
+  <dimension ref="A1:H611"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -16301,6 +16301,370 @@
       </c>
       <c r="H597" s="5">
         <v>739.74610499999994</v>
+      </c>
+    </row>
+    <row r="598" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A598" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B598" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C598" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D598" s="4">
+        <v>0.24456018518518499</v>
+      </c>
+      <c r="E598" s="4">
+        <v>0.29012731481481502</v>
+      </c>
+      <c r="F598" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G598" s="2">
+        <v>1</v>
+      </c>
+      <c r="H598" s="5">
+        <v>459.20778200000001</v>
+      </c>
+    </row>
+    <row r="599" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A599" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B599" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C599" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D599" s="4">
+        <v>0.29012731481481502</v>
+      </c>
+      <c r="E599" s="4">
+        <v>0.37502314814814802</v>
+      </c>
+      <c r="F599" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G599" s="2">
+        <v>1</v>
+      </c>
+      <c r="H599" s="5">
+        <v>867.59927700000003</v>
+      </c>
+    </row>
+    <row r="600" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A600" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B600" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C600" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D600" s="4">
+        <v>0.37502314814814802</v>
+      </c>
+      <c r="E600" s="4">
+        <v>0.50002314814814797</v>
+      </c>
+      <c r="F600" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G600" s="2">
+        <v>1</v>
+      </c>
+      <c r="H600" s="5">
+        <v>1441.304954</v>
+      </c>
+    </row>
+    <row r="601" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A601" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B601" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C601" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D601" s="4">
+        <v>0.50002314814814797</v>
+      </c>
+      <c r="E601" s="4">
+        <v>0.56252314814814797</v>
+      </c>
+      <c r="F601" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G601" s="2">
+        <v>1</v>
+      </c>
+      <c r="H601" s="5">
+        <v>1599.847925</v>
+      </c>
+    </row>
+    <row r="602" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A602" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B602" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C602" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D602" s="4">
+        <v>0.56252314814814797</v>
+      </c>
+      <c r="E602" s="4">
+        <v>0.60418981481481504</v>
+      </c>
+      <c r="F602" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G602" s="2">
+        <v>1</v>
+      </c>
+      <c r="H602" s="5">
+        <v>1487.415493</v>
+      </c>
+    </row>
+    <row r="603" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A603" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B603" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C603" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D603" s="4">
+        <v>0.60418981481481504</v>
+      </c>
+      <c r="E603" s="4">
+        <v>0.64583333333333304</v>
+      </c>
+      <c r="F603" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G603" s="2">
+        <v>1</v>
+      </c>
+      <c r="H603" s="5">
+        <v>1984.2137090000001</v>
+      </c>
+    </row>
+    <row r="604" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A604" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B604" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C604" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D604" s="4">
+        <v>0.64583333333333304</v>
+      </c>
+      <c r="E604" s="4">
+        <v>0.68753472222222201</v>
+      </c>
+      <c r="F604" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G604" s="2">
+        <v>1</v>
+      </c>
+      <c r="H604" s="5">
+        <v>2337.093969</v>
+      </c>
+    </row>
+    <row r="605" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A605" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B605" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C605" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D605" s="4">
+        <v>0.68753472222222201</v>
+      </c>
+      <c r="E605" s="4">
+        <v>0.770821759259259</v>
+      </c>
+      <c r="F605" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G605" s="2">
+        <v>1</v>
+      </c>
+      <c r="H605" s="5">
+        <v>2935.1661989999998</v>
+      </c>
+    </row>
+    <row r="606" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A606" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B606" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C606" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D606" s="4">
+        <v>0.770821759259259</v>
+      </c>
+      <c r="E606" s="4">
+        <v>0.81251157407407404</v>
+      </c>
+      <c r="F606" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G606" s="2">
+        <v>1</v>
+      </c>
+      <c r="H606" s="5">
+        <v>3398.039988</v>
+      </c>
+    </row>
+    <row r="607" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A607" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B607" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C607" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D607" s="4">
+        <v>0.81251157407407404</v>
+      </c>
+      <c r="E607" s="4">
+        <v>0.85421296296296301</v>
+      </c>
+      <c r="F607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G607" s="2">
+        <v>1</v>
+      </c>
+      <c r="H607" s="5">
+        <v>3941.4985710000001</v>
+      </c>
+    </row>
+    <row r="608" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A608" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B608" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C608" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D608" s="4">
+        <v>0.85421296296296301</v>
+      </c>
+      <c r="E608" s="4">
+        <v>0.89586805555555604</v>
+      </c>
+      <c r="F608" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G608" s="2">
+        <v>1</v>
+      </c>
+      <c r="H608" s="5">
+        <v>3854.8877149999998</v>
+      </c>
+    </row>
+    <row r="609" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A609" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B609" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C609" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D609" s="4">
+        <v>0.89586805555555604</v>
+      </c>
+      <c r="E609" s="4">
+        <v>0.93754629629629604</v>
+      </c>
+      <c r="F609" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G609" s="2">
+        <v>1</v>
+      </c>
+      <c r="H609" s="5">
+        <v>3780.1327999999999</v>
+      </c>
+    </row>
+    <row r="610" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A610" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B610" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C610" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D610" s="4">
+        <v>0.93754629629629604</v>
+      </c>
+      <c r="E610" s="4">
+        <v>0.963321759259259</v>
+      </c>
+      <c r="F610" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G610" s="2">
+        <v>1</v>
+      </c>
+      <c r="H610" s="5">
+        <v>2656.725719</v>
+      </c>
+    </row>
+    <row r="611" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A611" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B611" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C611" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D611" s="4">
+        <v>0.963321759259259</v>
+      </c>
+      <c r="E611" s="4">
+        <v>1.0053125000000001</v>
+      </c>
+      <c r="F611" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G611" s="2">
+        <v>1</v>
+      </c>
+      <c r="H611" s="5">
+        <v>961.78833899999995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reporte actualizado automaticamente el 2026-06-10
</commit_message>
<xml_diff>
--- a/Programmes Seguimiento LE_2.xlsx
+++ b/Programmes Seguimiento LE_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Seguimiento-LE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49814366-2DD2-42B3-8038-326E44BD50D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B4C41D-749B-4630-8529-DEB359F1060F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CON-Las Estrellas" sheetId="2" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="70">
   <si>
     <t>Targets</t>
   </si>
@@ -231,6 +231,9 @@
   </si>
   <si>
     <t xml:space="preserve">	 For Region [National] Universe 78427.2; Sample 6818 ( 100.00% )</t>
+  </si>
+  <si>
+    <t>HOY CELEBREMOS</t>
   </si>
 </sst>
 </file>
@@ -15908,7 +15911,7 @@
         <v>0.50002314814814797</v>
       </c>
       <c r="F582" s="2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="G582" s="2">
         <v>1</v>
@@ -16298,7 +16301,7 @@
         <v>0.50003472222222201</v>
       </c>
       <c r="F597" s="2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="G597" s="2">
         <v>1</v>

</xml_diff>